<commit_message>
initial commit (based on DEMO project)
</commit_message>
<xml_diff>
--- a/X-Series/XD12R/Reliability_BD/XD12R_GT1009A0R0_REL/Docs/jig_mcu_info.xlsx
+++ b/X-Series/XD12R/Reliability_BD/XD12R_GT1009A0R0_REL/Docs/jig_mcu_info.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\working\01_Project\Jig\XD_JIG\XD12\XD12R_GT1009A0R0\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\working\01_Project\FW\X-Series\XD12R\Demo_BD\XD12R_GT1009A0R0_DEMO\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9176BF98-F734-4CCC-B2A8-3F2C964BDE4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40940D79-7EE6-4F24-B8B3-C143709106BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="71880" yWindow="2160" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="38">
   <si>
     <t>TIM1</t>
     <phoneticPr fontId="18" type="noConversion"/>
@@ -125,14 +125,6 @@
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>xd data in</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>osc trim</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
     <t>us delay</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
@@ -151,14 +143,6 @@
     <t>SPI3</t>
   </si>
   <si>
-    <t>xc spi</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>adc spi</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
     <t>Peripheral</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
@@ -180,38 +164,6 @@
   </si>
   <si>
     <t>2 edge</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>xc</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>xd</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>MCLK</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>serial high</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>serial low</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>duty high</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>duty low</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>serial freq</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
@@ -227,10 +179,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="176" formatCode="0.0&quot;MHz&quot;"/>
     <numFmt numFmtId="177" formatCode="0.00&quot;MHz&quot;"/>
-    <numFmt numFmtId="178" formatCode="0.000&quot;MHz&quot;"/>
   </numFmts>
   <fonts count="19" x14ac:knownFonts="1">
     <font>
@@ -824,7 +775,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -835,9 +786,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -909,7 +857,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>31</xdr:col>
-      <xdr:colOff>524812</xdr:colOff>
+      <xdr:colOff>521637</xdr:colOff>
       <xdr:row>32</xdr:row>
       <xdr:rowOff>208188</xdr:rowOff>
     </xdr:to>
@@ -1274,10 +1222,10 @@
   <sheetData>
     <row r="2" spans="2:16" x14ac:dyDescent="0.45">
       <c r="C2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.45">
@@ -1445,25 +1393,19 @@
     </row>
     <row r="9" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B9" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C9" t="s">
         <v>24</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
+        <v>37</v>
+      </c>
+      <c r="J9" t="s">
+        <v>36</v>
+      </c>
+      <c r="N9" t="s">
         <v>25</v>
-      </c>
-      <c r="E9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G9" t="s">
-        <v>26</v>
-      </c>
-      <c r="J9" t="s">
-        <v>48</v>
-      </c>
-      <c r="N9" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="10" spans="2:16" x14ac:dyDescent="0.45">
@@ -1804,26 +1746,19 @@
         <v>90000000</v>
       </c>
     </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B18" s="1"/>
       <c r="C18" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.45">
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B19" s="1" t="s">
         <v>14</v>
       </c>
@@ -1836,17 +1771,8 @@
       <c r="E19" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G19" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="H19" s="3">
-        <v>16</v>
-      </c>
-      <c r="I19" s="4">
-        <v>39.319200000000002</v>
-      </c>
-    </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.45">
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B20" s="1" t="s">
         <v>23</v>
       </c>
@@ -1859,37 +1785,13 @@
       <c r="E20" s="1">
         <v>16</v>
       </c>
-      <c r="G20" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="H20">
-        <v>6</v>
-      </c>
-      <c r="I20">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.45">
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B21" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C21" t="s">
-        <v>32</v>
-      </c>
-      <c r="D21" t="s">
-        <v>33</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H21">
-        <v>10</v>
-      </c>
-      <c r="I21">
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B22" s="1" t="s">
         <v>17</v>
       </c>
@@ -1905,84 +1807,45 @@
         <f t="shared" si="3"/>
         <v>45</v>
       </c>
-      <c r="G22" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="H22">
-        <f>H20/(H20+H21)</f>
-        <v>0.375</v>
-      </c>
-      <c r="I22">
-        <f>I20/(I20+I21)</f>
-        <v>0.33333333333333331</v>
-      </c>
-    </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.45">
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B23" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C23">
-        <v>4</v>
-      </c>
-      <c r="D23">
-        <v>2</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="H23">
-        <f>H21/(H20+H21)</f>
-        <v>0.625</v>
-      </c>
-      <c r="I23">
-        <f>I21/(I20+I21)</f>
-        <v>0.66666666666666663</v>
-      </c>
-    </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.45">
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B24" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C24">
+      <c r="C24" t="e">
         <f>C22/(C23)</f>
-        <v>22.5</v>
-      </c>
-      <c r="D24">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D24" t="e">
         <f t="shared" ref="D24" si="4">D22/(D23)</f>
-        <v>22.5</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="H24">
-        <f>H19/(H20+H21)</f>
-        <v>1</v>
-      </c>
-      <c r="I24">
-        <f>I19/(I20+I21)</f>
-        <v>1.0081846153846155</v>
-      </c>
-    </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.45">
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B25" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C25" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D25" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.45">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B26" s="1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C26" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D26" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>